<commit_message>
Changed Push API logic
</commit_message>
<xml_diff>
--- a/pds_admin_bihar/Backend/Backend/Tagging_Sheet_Pre.xlsx
+++ b/pds_admin_bihar/Backend/Backend/Tagging_Sheet_Pre.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="23">
   <si>
     <t>Var</t>
   </si>
@@ -43,19 +43,46 @@
     <t>Araria</t>
   </si>
   <si>
+    <t>Pds</t>
+  </si>
+  <si>
     <t>Wheat</t>
   </si>
   <si>
-    <t>52.94</t>
-  </si>
-  <si>
-    <t>21.12</t>
-  </si>
-  <si>
-    <t>27.7</t>
-  </si>
-  <si>
-    <t>13.66</t>
+    <t>42.88</t>
+  </si>
+  <si>
+    <t>15.66</t>
+  </si>
+  <si>
+    <t>33.4</t>
+  </si>
+  <si>
+    <t>52.98</t>
+  </si>
+  <si>
+    <t>19.96</t>
+  </si>
+  <si>
+    <t>22.0</t>
+  </si>
+  <si>
+    <t>13.5</t>
+  </si>
+  <si>
+    <t>117.8</t>
+  </si>
+  <si>
+    <t>25.72</t>
+  </si>
+  <si>
+    <t>5.94</t>
+  </si>
+  <si>
+    <t>55.84</t>
+  </si>
+  <si>
+    <t>24.22</t>
   </si>
 </sst>
 </file>
@@ -413,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -453,16 +480,16 @@
         <v>8</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>120900100001</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -479,16 +506,16 @@
         <v>8</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>120900100004</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
       </c>
       <c r="G3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -505,16 +532,16 @@
         <v>8</v>
       </c>
       <c r="E4">
-        <v>8</v>
+        <v>120900100005</v>
       </c>
       <c r="F4" t="s">
         <v>8</v>
       </c>
       <c r="G4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -531,16 +558,250 @@
         <v>8</v>
       </c>
       <c r="E5">
+        <v>120900100006</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="1">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6">
+        <v>2030168</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>120900100007</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="1">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7">
+        <v>2030168</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>120900100008</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="1">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8">
+        <v>2030168</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8">
+        <v>120900100009</v>
+      </c>
+      <c r="F8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="1">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>2030168</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9">
+        <v>120900100012</v>
+      </c>
+      <c r="F9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="1">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10">
+        <v>2030168</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10">
+        <v>120900100013</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="1">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11">
+        <v>2030168</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11">
+        <v>120900100014</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="1">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12">
+        <v>2030168</v>
+      </c>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12">
+        <v>120900100015</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="1">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13">
+        <v>2030168</v>
+      </c>
+      <c r="D13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>121000000000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="1">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14">
+        <v>2030168</v>
+      </c>
+      <c r="D14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" t="s">
         <v>9</v>
       </c>
-      <c r="F5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H5" t="s">
-        <v>13</v>
+      <c r="F14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed frontend remaining issues
</commit_message>
<xml_diff>
--- a/pds_admin_bihar/Backend/Backend/Tagging_Sheet_Pre.xlsx
+++ b/pds_admin_bihar/Backend/Backend/Tagging_Sheet_Pre.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="36">
   <si>
     <t>Var</t>
   </si>
@@ -43,46 +43,85 @@
     <t>Araria</t>
   </si>
   <si>
-    <t>Pds</t>
+    <t>adminpds</t>
   </si>
   <si>
     <t>Wheat</t>
   </si>
   <si>
-    <t>42.88</t>
-  </si>
-  <si>
-    <t>15.66</t>
-  </si>
-  <si>
-    <t>33.4</t>
-  </si>
-  <si>
-    <t>52.98</t>
-  </si>
-  <si>
-    <t>19.96</t>
-  </si>
-  <si>
-    <t>22.0</t>
-  </si>
-  <si>
-    <t>13.5</t>
-  </si>
-  <si>
-    <t>117.8</t>
-  </si>
-  <si>
-    <t>25.72</t>
-  </si>
-  <si>
-    <t>5.94</t>
-  </si>
-  <si>
-    <t>55.84</t>
-  </si>
-  <si>
-    <t>24.22</t>
+    <t>44.2</t>
+  </si>
+  <si>
+    <t>28.29</t>
+  </si>
+  <si>
+    <t>16.72</t>
+  </si>
+  <si>
+    <t>33.68</t>
+  </si>
+  <si>
+    <t>63.24</t>
+  </si>
+  <si>
+    <t>21.12</t>
+  </si>
+  <si>
+    <t>27.7</t>
+  </si>
+  <si>
+    <t>13.66</t>
+  </si>
+  <si>
+    <t>46.78</t>
+  </si>
+  <si>
+    <t>26.5</t>
+  </si>
+  <si>
+    <t>6.56</t>
+  </si>
+  <si>
+    <t>53.6</t>
+  </si>
+  <si>
+    <t>49.75</t>
+  </si>
+  <si>
+    <t>25.88</t>
+  </si>
+  <si>
+    <t>0.35</t>
+  </si>
+  <si>
+    <t>120.0</t>
+  </si>
+  <si>
+    <t>52.94</t>
+  </si>
+  <si>
+    <t>47.25</t>
+  </si>
+  <si>
+    <t>51.7</t>
+  </si>
+  <si>
+    <t>68.02</t>
+  </si>
+  <si>
+    <t>29.94</t>
+  </si>
+  <si>
+    <t>27.76</t>
+  </si>
+  <si>
+    <t>17.04</t>
+  </si>
+  <si>
+    <t>18.72</t>
+  </si>
+  <si>
+    <t>12.38</t>
   </si>
 </sst>
 </file>
@@ -440,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -474,7 +513,7 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -500,13 +539,13 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3">
-        <v>120900100004</v>
+        <v>120900100002</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
@@ -526,13 +565,13 @@
         <v>7</v>
       </c>
       <c r="C4">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4">
-        <v>120900100005</v>
+        <v>120900100004</v>
       </c>
       <c r="F4" t="s">
         <v>8</v>
@@ -552,13 +591,13 @@
         <v>7</v>
       </c>
       <c r="C5">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
       </c>
       <c r="E5">
-        <v>120900100006</v>
+        <v>120900100005</v>
       </c>
       <c r="F5" t="s">
         <v>8</v>
@@ -578,13 +617,13 @@
         <v>7</v>
       </c>
       <c r="C6">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
       </c>
       <c r="E6">
-        <v>120900100007</v>
+        <v>120900100006</v>
       </c>
       <c r="F6" t="s">
         <v>8</v>
@@ -604,13 +643,13 @@
         <v>7</v>
       </c>
       <c r="C7">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7">
-        <v>120900100008</v>
+        <v>120900100007</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -630,13 +669,13 @@
         <v>7</v>
       </c>
       <c r="C8">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
       </c>
       <c r="E8">
-        <v>120900100009</v>
+        <v>120900100008</v>
       </c>
       <c r="F8" t="s">
         <v>8</v>
@@ -656,13 +695,13 @@
         <v>7</v>
       </c>
       <c r="C9">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D9" t="s">
         <v>8</v>
       </c>
       <c r="E9">
-        <v>120900100012</v>
+        <v>120900100009</v>
       </c>
       <c r="F9" t="s">
         <v>8</v>
@@ -682,13 +721,13 @@
         <v>7</v>
       </c>
       <c r="C10">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D10" t="s">
         <v>8</v>
       </c>
       <c r="E10">
-        <v>120900100013</v>
+        <v>120900100012</v>
       </c>
       <c r="F10" t="s">
         <v>8</v>
@@ -708,13 +747,13 @@
         <v>7</v>
       </c>
       <c r="C11">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D11" t="s">
         <v>8</v>
       </c>
       <c r="E11">
-        <v>120900100014</v>
+        <v>120900100013</v>
       </c>
       <c r="F11" t="s">
         <v>8</v>
@@ -734,13 +773,13 @@
         <v>7</v>
       </c>
       <c r="C12">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D12" t="s">
         <v>8</v>
       </c>
       <c r="E12">
-        <v>120900100015</v>
+        <v>120900100014</v>
       </c>
       <c r="F12" t="s">
         <v>8</v>
@@ -760,13 +799,13 @@
         <v>7</v>
       </c>
       <c r="C13">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D13" t="s">
         <v>8</v>
       </c>
       <c r="E13">
-        <v>121000000000</v>
+        <v>120900100015</v>
       </c>
       <c r="F13" t="s">
         <v>8</v>
@@ -775,7 +814,7 @@
         <v>10</v>
       </c>
       <c r="H13" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -786,22 +825,334 @@
         <v>7</v>
       </c>
       <c r="C14">
-        <v>2030168</v>
+        <v>2090130</v>
       </c>
       <c r="D14" t="s">
         <v>8</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14">
+        <v>120900100016</v>
+      </c>
+      <c r="F14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="1">
+        <v>26</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15">
+        <v>2090130</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15">
+        <v>120900100020</v>
+      </c>
+      <c r="F15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="1">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16">
+        <v>2090130</v>
+      </c>
+      <c r="D16" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16">
+        <v>120900100033</v>
+      </c>
+      <c r="F16" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="1">
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17">
+        <v>2090336</v>
+      </c>
+      <c r="D17" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" t="s">
         <v>9</v>
       </c>
-      <c r="F14" t="s">
-        <v>8</v>
-      </c>
-      <c r="G14" t="s">
-        <v>10</v>
-      </c>
-      <c r="H14" t="s">
-        <v>22</v>
+      <c r="F17" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="1">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18">
+        <v>2090375</v>
+      </c>
+      <c r="D18" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18">
+        <v>120900100010</v>
+      </c>
+      <c r="F18" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="1">
+        <v>34</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19">
+        <v>2090375</v>
+      </c>
+      <c r="D19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19">
+        <v>120900100025</v>
+      </c>
+      <c r="F19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="1">
+        <v>36</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20">
+        <v>2090375</v>
+      </c>
+      <c r="D20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20">
+        <v>120900100026</v>
+      </c>
+      <c r="F20" t="s">
+        <v>8</v>
+      </c>
+      <c r="G20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="1">
+        <v>38</v>
+      </c>
+      <c r="B21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21">
+        <v>2090375</v>
+      </c>
+      <c r="D21" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21">
+        <v>120900100029</v>
+      </c>
+      <c r="F21" t="s">
+        <v>8</v>
+      </c>
+      <c r="G21" t="s">
+        <v>10</v>
+      </c>
+      <c r="H21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="1">
+        <v>40</v>
+      </c>
+      <c r="B22" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22">
+        <v>2090375</v>
+      </c>
+      <c r="D22" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22">
+        <v>120900100030</v>
+      </c>
+      <c r="F22" t="s">
+        <v>8</v>
+      </c>
+      <c r="G22" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="1">
+        <v>42</v>
+      </c>
+      <c r="B23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23">
+        <v>2090375</v>
+      </c>
+      <c r="D23" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23">
+        <v>120900100031</v>
+      </c>
+      <c r="F23" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="1">
+        <v>44</v>
+      </c>
+      <c r="B24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24">
+        <v>2090375</v>
+      </c>
+      <c r="D24" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24">
+        <v>120900100032</v>
+      </c>
+      <c r="F24" t="s">
+        <v>8</v>
+      </c>
+      <c r="G24" t="s">
+        <v>10</v>
+      </c>
+      <c r="H24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="1">
+        <v>46</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25">
+        <v>2090375</v>
+      </c>
+      <c r="D25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25">
+        <v>120900100034</v>
+      </c>
+      <c r="F25" t="s">
+        <v>8</v>
+      </c>
+      <c r="G25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="1">
+        <v>48</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26">
+        <v>2090375</v>
+      </c>
+      <c r="D26" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26">
+        <v>120900100036</v>
+      </c>
+      <c r="F26" t="s">
+        <v>8</v>
+      </c>
+      <c r="G26" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>